<commit_message>
vault backup: 2026-07-03 10:42:17
</commit_message>
<xml_diff>
--- a/Daily-Task-List/Knowledge_Base/WTO-IOTC/WTO 渔业补贴条款历史演变示例表.xlsx
+++ b/Daily-Task-List/Knowledge_Base/WTO-IOTC/WTO 渔业补贴条款历史演变示例表.xlsx
@@ -1,13 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\1_Learning_Record\1_Typora\My-NoteBook\Daily-Task-List\Knowledge_Base\WTO-IOTC\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21D42D9A-967F-4267-80AF-7487233A96DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="版本1_W_20" sheetId="1" r:id="rId1"/>
+    <sheet name="版本2_W_5" sheetId="2" r:id="rId2"/>
+    <sheet name="版本3_W_276)" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -18,9 +26,152 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="29">
+  <si>
+    <t>字段</t>
+  </si>
+  <si>
+    <t>详细信息</t>
+  </si>
+  <si>
+    <t>条款内容</t>
+  </si>
+  <si>
+    <t>任何成员不得对捕鱼活动提供任何补贴。</t>
+  </si>
+  <si>
+    <t>修订动作</t>
+  </si>
+  <si>
+    <t>初始草案</t>
+  </si>
+  <si>
+    <t>主要提案方</t>
+  </si>
+  <si>
+    <t>主席</t>
+  </si>
+  <si>
+    <t>支持方</t>
+  </si>
+  <si>
+    <t>全体</t>
+  </si>
+  <si>
+    <t>反对方</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>修订理由</t>
+  </si>
+  <si>
+    <t>作为谈判的基准文本。</t>
+  </si>
+  <si>
+    <t>当前动作</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>初始草案</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>提案方</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>主席</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>任何成员不得对捕鱼活动提供任何补贴，</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>发展中国家除外。</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>确保小规模手工渔民的生计和粮食安全。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>非洲集团、最不发达国家</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>印度</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>增加例外条款</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>将重点转向最具破坏性的捕鱼行为，保护合法的远洋船队。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>美国</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>日本、韩国</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>欧盟</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>缩小禁令范围</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>任何成员不得对</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>非法、不报告和不管制（IUU）的</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>捕鱼活动提供任何补贴，发展中国家除外。</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -28,13 +179,43 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="2"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,11 +230,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -330,10 +517,262 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="64.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7166255C-F99B-4B15-8597-05A1F62DF7A4}">
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="55.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="28" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DBB1B42-121B-4B09-9D1C-148D14FCB9EF}">
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="81.25" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
vault backup: 2026-07-03 10:46:40
</commit_message>
<xml_diff>
--- a/Daily-Task-List/Knowledge_Base/WTO-IOTC/WTO 渔业补贴条款历史演变示例表.xlsx
+++ b/Daily-Task-List/Knowledge_Base/WTO-IOTC/WTO 渔业补贴条款历史演变示例表.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\1_Learning_Record\1_Typora\My-NoteBook\Daily-Task-List\Knowledge_Base\WTO-IOTC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21D42D9A-967F-4267-80AF-7487233A96DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F96AA3C9-EA0B-4A1A-8271-7511BEB8272F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="版本1_W_20" sheetId="1" r:id="rId1"/>
     <sheet name="版本2_W_5" sheetId="2" r:id="rId2"/>
     <sheet name="版本3_W_276)" sheetId="3" r:id="rId3"/>
+    <sheet name="版本4_W_285" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="35">
   <si>
     <t>字段</t>
   </si>
@@ -163,6 +164,53 @@
         <scheme val="minor"/>
       </rPr>
       <t>捕鱼活动提供任何补贴，发展中国家除外。</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>限制例外范围</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>主席 (折中方案)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>防止公海补贴漏洞，达成最终妥协。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>-</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>多数成员（共识）</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>任何成员不得对非法、不报告和不管制（IUU）的捕鱼活动提供任何补贴，</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>其专属经济区（EEZ）内</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>的发展中国家除外。</t>
     </r>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -760,7 +808,7 @@
         <v>14</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
@@ -768,7 +816,94 @@
         <v>16</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>21</v>
+        <v>26</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC16B71F-C2BA-499F-97EF-F0044E3ABDB3}">
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="81.25" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="28" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>